<commit_message>
Tableau de synthèse E5 : lignes alternance
</commit_message>
<xml_diff>
--- a/documents/tableau-synthese-E5-Fourier-Tiago.xlsx
+++ b/documents/tableau-synthese-E5-Fourier-Tiago.xlsx
@@ -1449,23 +1449,49 @@
       <c r="H27" s="54" t="n"/>
     </row>
     <row r="28" ht="39.75" customHeight="1" s="43">
-      <c r="A28" s="56" t="inlineStr"/>
-      <c r="B28" s="57" t="inlineStr"/>
-      <c r="C28" s="59" t="n"/>
+      <c r="A28" s="56" t="inlineStr">
+        <is>
+          <t>serveur de téléphonie IP Wazo Platform pour LOXYS : VM Debian 12, wazo-ansible, softphones de test, agent Zabbix</t>
+        </is>
+      </c>
+      <c r="B28" s="57" t="inlineStr">
+        <is>
+          <t>oct. 2026</t>
+        </is>
+      </c>
+      <c r="C28" s="32" t="n">
+        <v>4</v>
+      </c>
       <c r="D28" s="26" t="n"/>
       <c r="E28" s="26" t="n"/>
       <c r="F28" s="26" t="n"/>
-      <c r="G28" s="26" t="n"/>
+      <c r="G28" s="32" t="inlineStr">
+        <is>
+          <t>1 - 2</t>
+        </is>
+      </c>
       <c r="H28" s="28" t="n"/>
     </row>
     <row r="29" ht="39.75" customHeight="1" s="43">
-      <c r="A29" s="56" t="inlineStr"/>
-      <c r="B29" s="57" t="inlineStr"/>
+      <c r="A29" s="56" t="inlineStr">
+        <is>
+          <t>support utilisateurs et dépannage de PC (1 à 3 interventions par jour), WiFi du festival The N'Joy</t>
+        </is>
+      </c>
+      <c r="B29" s="57" t="inlineStr">
+        <is>
+          <t>depuis le 01/09/26</t>
+        </is>
+      </c>
       <c r="C29" s="59" t="n"/>
-      <c r="D29" s="26" t="n"/>
+      <c r="D29" s="32" t="n">
+        <v>2</v>
+      </c>
       <c r="E29" s="26" t="n"/>
       <c r="F29" s="26" t="n"/>
-      <c r="G29" s="26" t="n"/>
+      <c r="G29" s="32" t="n">
+        <v>2</v>
+      </c>
       <c r="H29" s="28" t="n"/>
     </row>
     <row r="30" ht="19.5" customHeight="1" s="43">
@@ -11307,13 +11333,15 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A24" r:id="rId23"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A25" r:id="rId24"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A26" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A31" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A32" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A33" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A35" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A36" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A37" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A38" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A28" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A29" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A31" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A32" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A33" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A35" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A36" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A37" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A38" r:id="rId34"/>
   </hyperlinks>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.1968503937007874" right="0.1968503937007874" top="0.1968503937007874" bottom="0.1968503937007874" header="0" footer="0"/>

</xml_diff>